<commit_message>
data: 美股 2016~2025 財務更新
</commit_message>
<xml_diff>
--- a/data/美股_10年財務.xlsx
+++ b/data/美股_10年財務.xlsx
@@ -3820,12 +3820,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>RMD</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ResMed Inc.</t>
+          <t>Exelixis, Inc.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3839,7 +3839,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F38" t="n">
         <v>2016</v>
@@ -3848,80 +3848,80 @@
         <v>2025</v>
       </c>
       <c r="H38" t="n">
-        <v>18.4</v>
+        <v>1.9</v>
       </c>
       <c r="I38" t="n">
-        <v>51.5</v>
+        <v>23.2</v>
       </c>
       <c r="J38" t="n">
-        <v>14</v>
+        <v>7.8</v>
       </c>
       <c r="K38" t="n">
-        <v>16.6</v>
+        <v>8.4</v>
       </c>
       <c r="L38" t="n">
-        <v>3.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>9.300000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="N38" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="n">
-        <v>11.7</v>
+        <v>18.6</v>
       </c>
       <c r="Q38" t="n">
         <v>12.9</v>
       </c>
       <c r="R38" t="n">
-        <v>9.800000000000001</v>
+        <v>7</v>
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="n">
-        <v>17.6</v>
+        <v>47.6</v>
       </c>
       <c r="U38" t="n">
-        <v>21.6</v>
+        <v>62.5</v>
       </c>
       <c r="V38" t="n">
-        <v>37.2</v>
+        <v>50.1</v>
       </c>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="n">
-        <v>19</v>
+        <v>36.4</v>
       </c>
       <c r="Y38" t="n">
-        <v>104.2</v>
+        <v>55.6</v>
       </c>
       <c r="Z38" t="n">
-        <v>29.2</v>
+        <v>33.2</v>
       </c>
       <c r="AA38" t="n">
-        <v>27.2</v>
+        <v>33.7</v>
       </c>
       <c r="AB38" t="n">
-        <v>8</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AC38" t="n">
-        <v>119</v>
+        <v>108</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>RMD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Salesforce, Inc.</t>
+          <t>ResMed Inc.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3930,7 +3930,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F39" t="n">
         <v>2016</v>
@@ -3939,80 +3939,80 @@
         <v>2025</v>
       </c>
       <c r="H39" t="n">
-        <v>66.7</v>
+        <v>18.4</v>
       </c>
       <c r="I39" t="n">
-        <v>378.9</v>
+        <v>51.5</v>
       </c>
       <c r="J39" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="K39" t="n">
-        <v>124.3</v>
+        <v>16.6</v>
       </c>
       <c r="L39" t="n">
-        <v>54.9</v>
+        <v>3.3</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>40.6</v>
+        <v>27</v>
       </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="n">
-        <v>17.3</v>
+        <v>11.7</v>
       </c>
       <c r="Q39" t="n">
-        <v>12.7</v>
+        <v>12.9</v>
       </c>
       <c r="R39" t="n">
-        <v>8.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="n">
-        <v>118</v>
+        <v>17.6</v>
       </c>
       <c r="U39" t="n">
-        <v>62.5</v>
+        <v>21.6</v>
       </c>
       <c r="V39" t="n">
-        <v>49.8</v>
+        <v>37.2</v>
       </c>
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="n">
-        <v>27.5</v>
+        <v>19</v>
       </c>
       <c r="Y39" t="n">
-        <v>33</v>
+        <v>104.2</v>
       </c>
       <c r="Z39" t="n">
-        <v>30.9</v>
+        <v>29.2</v>
       </c>
       <c r="AA39" t="n">
-        <v>16.4</v>
+        <v>27.2</v>
       </c>
       <c r="AB39" t="n">
-        <v>17.1</v>
+        <v>8</v>
       </c>
       <c r="AC39" t="n">
-        <v>201</v>
+        <v>119</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Netflix, Inc.</t>
+          <t>Salesforce, Inc.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F40" t="n">
         <v>2016</v>
@@ -4030,75 +4030,75 @@
         <v>2025</v>
       </c>
       <c r="H40" t="n">
-        <v>88.3</v>
+        <v>66.7</v>
       </c>
       <c r="I40" t="n">
-        <v>451.8</v>
+        <v>378.9</v>
       </c>
       <c r="J40" t="n">
-        <v>109.8</v>
+        <v>62</v>
       </c>
       <c r="K40" t="n">
-        <v>94.59999999999999</v>
+        <v>124.3</v>
       </c>
       <c r="L40" t="n">
-        <v>33.9</v>
+        <v>54.9</v>
       </c>
       <c r="M40" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>52.1</v>
+        <v>40.6</v>
       </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="n">
-        <v>12.6</v>
+        <v>17.3</v>
       </c>
       <c r="Q40" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="R40" t="n">
-        <v>15.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="n">
-        <v>31.8</v>
+        <v>118</v>
       </c>
       <c r="U40" t="n">
-        <v>34.7</v>
+        <v>62.5</v>
       </c>
       <c r="V40" t="n">
-        <v>26.1</v>
+        <v>49.8</v>
       </c>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="n">
-        <v>37.4</v>
+        <v>27.5</v>
       </c>
       <c r="Y40" t="n">
-        <v>80.09999999999999</v>
+        <v>33</v>
       </c>
       <c r="Z40" t="n">
-        <v>36.7</v>
+        <v>30.9</v>
       </c>
       <c r="AA40" t="n">
-        <v>24.3</v>
+        <v>16.4</v>
       </c>
       <c r="AB40" t="n">
-        <v>22.2</v>
+        <v>17.1</v>
       </c>
       <c r="AC40" t="n">
-        <v>86</v>
+        <v>201</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
+          <t>Netflix, Inc.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F41" t="n">
         <v>2016</v>
@@ -4121,80 +4121,80 @@
         <v>2025</v>
       </c>
       <c r="H41" t="n">
-        <v>902.7</v>
+        <v>88.3</v>
       </c>
       <c r="I41" t="n">
-        <v>4029.6</v>
+        <v>451.8</v>
       </c>
       <c r="J41" t="n">
-        <v>1321.7</v>
+        <v>109.8</v>
       </c>
       <c r="K41" t="n">
-        <v>732.7</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="L41" t="n">
-        <v>610.9</v>
+        <v>33.9</v>
       </c>
       <c r="M41" t="n">
         <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>30.2</v>
+        <v>52.1</v>
       </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="n">
-        <v>17.2</v>
+        <v>12.6</v>
       </c>
       <c r="Q41" t="n">
-        <v>12.5</v>
+        <v>12.6</v>
       </c>
       <c r="R41" t="n">
-        <v>15.1</v>
+        <v>15.9</v>
       </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="n">
-        <v>26.8</v>
+        <v>31.8</v>
       </c>
       <c r="U41" t="n">
-        <v>30.1</v>
+        <v>34.7</v>
       </c>
       <c r="V41" t="n">
-        <v>32</v>
+        <v>26.1</v>
       </c>
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="n">
-        <v>11.3</v>
+        <v>37.4</v>
       </c>
       <c r="Y41" t="n">
-        <v>6.9</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="Z41" t="n">
-        <v>0.7</v>
+        <v>36.7</v>
       </c>
       <c r="AA41" t="n">
-        <v>32.8</v>
+        <v>24.3</v>
       </c>
       <c r="AB41" t="n">
-        <v>11.2</v>
+        <v>22.2</v>
       </c>
       <c r="AC41" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -4212,80 +4212,80 @@
         <v>2025</v>
       </c>
       <c r="H42" t="n">
-        <v>911.5</v>
+        <v>902.7</v>
       </c>
       <c r="I42" t="n">
-        <v>2817.2</v>
+        <v>4029.6</v>
       </c>
       <c r="J42" t="n">
-        <v>1018.3</v>
+        <v>1321.7</v>
       </c>
       <c r="K42" t="n">
-        <v>716.1</v>
+        <v>732.7</v>
       </c>
       <c r="L42" t="n">
-        <v>324.9</v>
+        <v>610.9</v>
       </c>
       <c r="M42" t="n">
-        <v>9.4</v>
+        <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>44.5</v>
+        <v>30.2</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="n">
-        <v>14.5</v>
+        <v>17.2</v>
       </c>
       <c r="Q42" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="R42" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="n">
-        <v>18.1</v>
+        <v>26.8</v>
       </c>
       <c r="U42" t="n">
-        <v>11.9</v>
+        <v>30.1</v>
       </c>
       <c r="V42" t="n">
-        <v>15.5</v>
+        <v>32</v>
       </c>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="n">
-        <v>9.6</v>
+        <v>11.3</v>
       </c>
       <c r="Y42" t="n">
-        <v>3.2</v>
+        <v>6.9</v>
       </c>
       <c r="Z42" t="n">
-        <v>-3.3</v>
+        <v>0.7</v>
       </c>
       <c r="AA42" t="n">
-        <v>36.1</v>
+        <v>32.8</v>
       </c>
       <c r="AB42" t="n">
-        <v>13.6</v>
+        <v>11.2</v>
       </c>
       <c r="AC42" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Ferrari N.V.</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4303,80 +4303,80 @@
         <v>2025</v>
       </c>
       <c r="H43" t="n">
-        <v>31.1</v>
+        <v>911.5</v>
       </c>
       <c r="I43" t="n">
-        <v>71.5</v>
+        <v>2817.2</v>
       </c>
       <c r="J43" t="n">
-        <v>16</v>
+        <v>1018.3</v>
       </c>
       <c r="K43" t="n">
-        <v>26.6</v>
+        <v>716.1</v>
       </c>
       <c r="L43" t="n">
-        <v>9.199999999999999</v>
+        <v>324.9</v>
       </c>
       <c r="M43" t="n">
-        <v>11.1</v>
+        <v>9.4</v>
       </c>
       <c r="N43" t="n">
-        <v>59.3</v>
+        <v>44.5</v>
       </c>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="n">
-        <v>15.6</v>
+        <v>14.5</v>
       </c>
       <c r="Q43" t="n">
-        <v>11.9</v>
+        <v>12.4</v>
       </c>
       <c r="R43" t="n">
-        <v>7</v>
+        <v>14.9</v>
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="n">
-        <v>21.3</v>
+        <v>18.1</v>
       </c>
       <c r="U43" t="n">
-        <v>19.6</v>
+        <v>11.9</v>
       </c>
       <c r="V43" t="n">
-        <v>4.9</v>
+        <v>15.5</v>
       </c>
       <c r="W43" t="inlineStr"/>
       <c r="X43" t="n">
-        <v>83.09999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="Y43" t="n">
-        <v>64.3</v>
+        <v>3.2</v>
       </c>
       <c r="Z43" t="n">
-        <v>183.5</v>
+        <v>-3.3</v>
       </c>
       <c r="AA43" t="n">
-        <v>22.3</v>
+        <v>36.1</v>
       </c>
       <c r="AB43" t="n">
-        <v>9.5</v>
+        <v>13.6</v>
       </c>
       <c r="AC43" t="n">
-        <v>166</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Autodesk, Inc.</t>
+          <t>Ferrari N.V.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4394,89 +4394,89 @@
         <v>2025</v>
       </c>
       <c r="H44" t="n">
-        <v>25</v>
+        <v>31.1</v>
       </c>
       <c r="I44" t="n">
-        <v>61.3</v>
+        <v>71.5</v>
       </c>
       <c r="J44" t="n">
+        <v>16</v>
+      </c>
+      <c r="K44" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="L44" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="M44" t="n">
         <v>11.1</v>
       </c>
-      <c r="K44" t="n">
-        <v>15.1</v>
-      </c>
-      <c r="L44" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="M44" t="n">
-        <v>0</v>
-      </c>
       <c r="N44" t="n">
-        <v>75.8</v>
+        <v>59.3</v>
       </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="n">
-        <v>13.4</v>
+        <v>15.6</v>
       </c>
       <c r="Q44" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R44" t="n">
-        <v>11.5</v>
+        <v>7</v>
       </c>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="n">
-        <v>39</v>
+        <v>21.3</v>
       </c>
       <c r="U44" t="n">
-        <v>30.8</v>
+        <v>19.6</v>
       </c>
       <c r="V44" t="n">
-        <v>22.7</v>
+        <v>4.9</v>
       </c>
       <c r="W44" t="inlineStr"/>
       <c r="X44" t="n">
-        <v>2</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.9</v>
+        <v>64.3</v>
       </c>
       <c r="Z44" t="n">
-        <v>17.4</v>
+        <v>183.5</v>
       </c>
       <c r="AA44" t="n">
-        <v>18.1</v>
+        <v>22.3</v>
       </c>
       <c r="AB44" t="n">
-        <v>31.3</v>
+        <v>9.5</v>
       </c>
       <c r="AC44" t="n">
-        <v>135</v>
+        <v>166</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
+          <t>Autodesk, Inc.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="F45" t="n">
         <v>2016</v>
@@ -4485,85 +4485,89 @@
         <v>2025</v>
       </c>
       <c r="H45" t="n">
-        <v>1359.9</v>
+        <v>25</v>
       </c>
       <c r="I45" t="n">
-        <v>7169.2</v>
+        <v>61.3</v>
       </c>
       <c r="J45" t="n">
-        <v>776.7</v>
+        <v>11.1</v>
       </c>
       <c r="K45" t="n">
-        <v>77</v>
+        <v>15.1</v>
       </c>
       <c r="L45" t="n">
-        <v>1085.2</v>
+        <v>14.8</v>
       </c>
       <c r="M45" t="n">
-        <v>383.2</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>49.8</v>
+        <v>75.8</v>
       </c>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="Q45" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="R45" t="n">
-        <v>12.4</v>
+        <v>11.5</v>
       </c>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="U45" t="inlineStr"/>
+        <v>39</v>
+      </c>
+      <c r="U45" t="n">
+        <v>30.8</v>
+      </c>
       <c r="V45" t="n">
-        <v>31.1</v>
+        <v>22.7</v>
       </c>
       <c r="W45" t="inlineStr"/>
       <c r="X45" t="n">
-        <v>-21.6</v>
-      </c>
-      <c r="Y45" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>0.9</v>
+      </c>
       <c r="Z45" t="n">
-        <v>-76.59999999999999</v>
+        <v>17.4</v>
       </c>
       <c r="AA45" t="n">
-        <v>10.8</v>
+        <v>18.1</v>
       </c>
       <c r="AB45" t="n">
-        <v>9.1</v>
+        <v>31.3</v>
       </c>
       <c r="AC45" t="n">
-        <v>10</v>
+        <v>135</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Qualys, Inc.</t>
+          <t>Amazon.com, Inc.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="F46" t="n">
         <v>2016</v>
@@ -4572,80 +4576,76 @@
         <v>2025</v>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>1359.9</v>
       </c>
       <c r="I46" t="n">
-        <v>6.7</v>
+        <v>7169.2</v>
       </c>
       <c r="J46" t="n">
-        <v>2</v>
+        <v>776.7</v>
       </c>
       <c r="K46" t="n">
-        <v>3</v>
+        <v>77</v>
       </c>
       <c r="L46" t="n">
-        <v>1.2</v>
+        <v>1085.2</v>
       </c>
       <c r="M46" t="n">
-        <v>0</v>
+        <v>383.2</v>
       </c>
       <c r="N46" t="n">
-        <v>48.8</v>
+        <v>49.8</v>
       </c>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="Q46" t="n">
-        <v>11</v>
+        <v>11.7</v>
       </c>
       <c r="R46" t="n">
-        <v>10.1</v>
+        <v>12.4</v>
       </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="U46" t="n">
-        <v>22.5</v>
-      </c>
+        <v>29.5</v>
+      </c>
+      <c r="U46" t="inlineStr"/>
       <c r="V46" t="n">
-        <v>14.2</v>
+        <v>31.1</v>
       </c>
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="Y46" t="n">
-        <v>20.3</v>
-      </c>
+        <v>-21.6</v>
+      </c>
+      <c r="Y46" t="inlineStr"/>
       <c r="Z46" t="n">
-        <v>31.3</v>
+        <v>-76.59999999999999</v>
       </c>
       <c r="AA46" t="n">
-        <v>29.6</v>
+        <v>10.8</v>
       </c>
       <c r="AB46" t="n">
-        <v>19.9</v>
+        <v>9.1</v>
       </c>
       <c r="AC46" t="n">
-        <v>153</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>QLYS</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Visa Inc.</t>
+          <t>Qualys, Inc.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4654,7 +4654,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F47" t="n">
         <v>2016</v>
@@ -4663,89 +4663,89 @@
         <v>2025</v>
       </c>
       <c r="H47" t="n">
-        <v>150.8</v>
+        <v>2</v>
       </c>
       <c r="I47" t="n">
-        <v>400</v>
+        <v>6.7</v>
       </c>
       <c r="J47" t="n">
-        <v>200.6</v>
+        <v>2</v>
       </c>
       <c r="K47" t="n">
-        <v>215.8</v>
+        <v>3</v>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="M47" t="n">
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>61.9</v>
+        <v>48.8</v>
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="n">
-        <v>12.9</v>
+        <v>13</v>
       </c>
       <c r="Q47" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="R47" t="n">
-        <v>11.3</v>
+        <v>10.1</v>
       </c>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="n">
-        <v>13</v>
+        <v>16.7</v>
       </c>
       <c r="U47" t="n">
-        <v>10.3</v>
+        <v>22.5</v>
       </c>
       <c r="V47" t="n">
-        <v>1.6</v>
+        <v>14.2</v>
       </c>
       <c r="W47" t="inlineStr"/>
       <c r="X47" t="n">
-        <v>17.3</v>
+        <v>15.2</v>
       </c>
       <c r="Y47" t="n">
-        <v>6.5</v>
+        <v>20.3</v>
       </c>
       <c r="Z47" t="n">
-        <v>15.4</v>
+        <v>31.3</v>
       </c>
       <c r="AA47" t="n">
-        <v>50.1</v>
+        <v>29.6</v>
       </c>
       <c r="AB47" t="n">
-        <v>10.4</v>
+        <v>19.9</v>
       </c>
       <c r="AC47" t="n">
-        <v>108</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>NICE</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>NICE Ltd.</t>
+          <t>Visa Inc.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="F48" t="n">
         <v>2016</v>
@@ -4754,64 +4754,64 @@
         <v>2025</v>
       </c>
       <c r="H48" t="n">
-        <v>10.2</v>
+        <v>150.8</v>
       </c>
       <c r="I48" t="n">
-        <v>29.5</v>
+        <v>400</v>
       </c>
       <c r="J48" t="n">
-        <v>6.1</v>
+        <v>200.6</v>
       </c>
       <c r="K48" t="n">
-        <v>7</v>
+        <v>215.8</v>
       </c>
       <c r="L48" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="M48" t="n">
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>24.1</v>
+        <v>61.9</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
-        <v>12.3</v>
+        <v>12.9</v>
       </c>
       <c r="Q48" t="n">
-        <v>10.5</v>
+        <v>10.9</v>
       </c>
       <c r="R48" t="n">
-        <v>7.7</v>
+        <v>11.3</v>
       </c>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="n">
-        <v>25.5</v>
+        <v>13</v>
       </c>
       <c r="U48" t="n">
-        <v>32</v>
+        <v>10.3</v>
       </c>
       <c r="V48" t="n">
-        <v>38.3</v>
+        <v>1.6</v>
       </c>
       <c r="W48" t="inlineStr"/>
       <c r="X48" t="n">
-        <v>11</v>
+        <v>17.3</v>
       </c>
       <c r="Y48" t="n">
-        <v>20.9</v>
+        <v>6.5</v>
       </c>
       <c r="Z48" t="n">
-        <v>-4.1</v>
+        <v>15.4</v>
       </c>
       <c r="AA48" t="n">
-        <v>20.8</v>
+        <v>50.1</v>
       </c>
       <c r="AB48" t="n">
-        <v>9.300000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="AC48" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="49">
@@ -4908,26 +4908,26 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>NICE</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Exelixis, Inc.</t>
+          <t>NICE Ltd.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="F50" t="n">
         <v>2016</v>
@@ -4936,58 +4936,64 @@
         <v>2025</v>
       </c>
       <c r="H50" t="n">
-        <v>1.9</v>
+        <v>10.2</v>
       </c>
       <c r="I50" t="n">
-        <v>21.7</v>
+        <v>29.5</v>
       </c>
       <c r="J50" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
       <c r="K50" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
       <c r="L50" t="n">
-        <v>9.1</v>
+        <v>3.6</v>
       </c>
       <c r="M50" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>23.9</v>
+        <v>24.1</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="n">
-        <v>17</v>
+        <v>12.3</v>
       </c>
       <c r="Q50" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="R50" t="inlineStr"/>
+        <v>10.5</v>
+      </c>
+      <c r="R50" t="n">
+        <v>7.7</v>
+      </c>
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="n">
-        <v>36.1</v>
+        <v>25.5</v>
       </c>
       <c r="U50" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="V50" t="inlineStr"/>
+        <v>32</v>
+      </c>
+      <c r="V50" t="n">
+        <v>38.3</v>
+      </c>
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="n">
-        <v>28.8</v>
+        <v>11</v>
       </c>
       <c r="Y50" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="Z50" t="inlineStr"/>
+        <v>20.9</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>-4.1</v>
+      </c>
       <c r="AA50" t="n">
-        <v>24</v>
+        <v>20.8</v>
       </c>
       <c r="AB50" t="n">
-        <v>60.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AC50" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="51">
@@ -10504,9 +10510,11 @@
       <c r="J35" t="n">
         <v>18.3</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>21.7</v>
+      </c>
       <c r="L35" t="n">
-        <v>21.7</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="36">
@@ -14496,9 +14504,11 @@
       <c r="J35" t="n">
         <v>2.1</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>5.2</v>
+      </c>
       <c r="L35" t="n">
-        <v>5.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="36">
@@ -18488,9 +18498,11 @@
       <c r="J35" t="n">
         <v>1.7</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>6.3</v>
+      </c>
       <c r="L35" t="n">
-        <v>6.3</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="36">
@@ -22480,9 +22492,11 @@
       <c r="J35" t="n">
         <v>10.4</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>9.1</v>
+      </c>
       <c r="L35" t="n">
-        <v>9.1</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="36">
@@ -26472,7 +26486,9 @@
       <c r="J35" t="n">
         <v>0.2</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>0.2</v>
+      </c>
       <c r="L35" t="n">
         <v>0.2</v>
       </c>
@@ -30466,9 +30482,11 @@
       <c r="J35" t="n">
         <v>23.1</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>23.9</v>
+      </c>
       <c r="L35" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36">

</xml_diff>